<commit_message>
Importing Data form excel to python + Defining function for implementing 3 different architecture on our data
</commit_message>
<xml_diff>
--- a/Data.xlsx
+++ b/Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Kashan University\Semester 8\Machine Learning\ML Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{539D6DD5-B26E-4D06-A0AF-D56DB642D0C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFE2DDE1-398D-413F-9B97-1D49415038C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,10 +36,10 @@
     <t>Attendence</t>
   </si>
   <si>
-    <t xml:space="preserve">Assignment </t>
+    <t xml:space="preserve">Pass </t>
   </si>
   <si>
-    <t xml:space="preserve">Pass </t>
+    <t xml:space="preserve">homework </t>
   </si>
 </sst>
 </file>
@@ -360,7 +360,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.77734375" customWidth="1"/>
@@ -378,11 +378,11 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -390,16 +390,16 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="C2">
-        <v>98</v>
+        <v>60</v>
       </c>
       <c r="D2">
-        <v>56</v>
+        <v>40</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -407,13 +407,13 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>11</v>
+        <v>42</v>
       </c>
       <c r="C3">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D3">
-        <v>67</v>
+        <v>45</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -424,16 +424,16 @@
         <v>1</v>
       </c>
       <c r="B4">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="C4">
-        <v>33</v>
+        <v>55</v>
       </c>
       <c r="D4">
-        <v>78</v>
+        <v>35</v>
       </c>
       <c r="E4">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -441,13 +441,13 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>5</v>
+        <v>50</v>
       </c>
       <c r="C5">
-        <v>89</v>
+        <v>70</v>
       </c>
       <c r="D5">
-        <v>89</v>
+        <v>50</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -458,13 +458,13 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>8</v>
+        <v>55</v>
       </c>
       <c r="C6">
-        <v>32</v>
+        <v>75</v>
       </c>
       <c r="D6">
-        <v>12</v>
+        <v>60</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -475,16 +475,832 @@
         <v>6</v>
       </c>
       <c r="B7">
+        <v>60</v>
+      </c>
+      <c r="C7">
+        <v>80</v>
+      </c>
+      <c r="D7">
+        <v>65</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8">
         <v>7</v>
       </c>
-      <c r="C7">
-        <v>11</v>
-      </c>
-      <c r="D7">
+      <c r="B8">
+        <v>68</v>
+      </c>
+      <c r="C8">
+        <v>85</v>
+      </c>
+      <c r="D8">
+        <v>70</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>75</v>
+      </c>
+      <c r="C9">
         <v>90</v>
       </c>
-      <c r="E7">
-        <v>0</v>
+      <c r="D9">
+        <v>80</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>2</v>
+      </c>
+      <c r="B10">
+        <v>45</v>
+      </c>
+      <c r="C10">
+        <v>80</v>
+      </c>
+      <c r="D10">
+        <v>55</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>3</v>
+      </c>
+      <c r="B11">
+        <v>52</v>
+      </c>
+      <c r="C11">
+        <v>78</v>
+      </c>
+      <c r="D11">
+        <v>60</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>4</v>
+      </c>
+      <c r="B12">
+        <v>48</v>
+      </c>
+      <c r="C12">
+        <v>82</v>
+      </c>
+      <c r="D12">
+        <v>58</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>5</v>
+      </c>
+      <c r="B13">
+        <v>65</v>
+      </c>
+      <c r="C13">
+        <v>70</v>
+      </c>
+      <c r="D13">
+        <v>72</v>
+      </c>
+      <c r="E13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>6</v>
+      </c>
+      <c r="B14">
+        <v>58</v>
+      </c>
+      <c r="C14">
+        <v>60</v>
+      </c>
+      <c r="D14">
+        <v>65</v>
+      </c>
+      <c r="E14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>1</v>
+      </c>
+      <c r="B15">
+        <v>25</v>
+      </c>
+      <c r="C15">
+        <v>50</v>
+      </c>
+      <c r="D15">
+        <v>30</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>9</v>
+      </c>
+      <c r="B16">
+        <v>88</v>
+      </c>
+      <c r="C16">
+        <v>95</v>
+      </c>
+      <c r="D16">
+        <v>92</v>
+      </c>
+      <c r="E16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>10</v>
+      </c>
+      <c r="B17">
+        <v>92</v>
+      </c>
+      <c r="C17">
+        <v>96</v>
+      </c>
+      <c r="D17">
+        <v>95</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>8</v>
+      </c>
+      <c r="B18">
+        <v>80</v>
+      </c>
+      <c r="C18">
+        <v>88</v>
+      </c>
+      <c r="D18">
+        <v>84</v>
+      </c>
+      <c r="E18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>7</v>
+      </c>
+      <c r="B19">
+        <v>72</v>
+      </c>
+      <c r="C19">
+        <v>84</v>
+      </c>
+      <c r="D19">
+        <v>76</v>
+      </c>
+      <c r="E19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>3</v>
+      </c>
+      <c r="B20">
+        <v>40</v>
+      </c>
+      <c r="C20">
+        <v>68</v>
+      </c>
+      <c r="D20">
+        <v>48</v>
+      </c>
+      <c r="E20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>4</v>
+      </c>
+      <c r="B21">
+        <v>55</v>
+      </c>
+      <c r="C21">
+        <v>74</v>
+      </c>
+      <c r="D21">
+        <v>60</v>
+      </c>
+      <c r="E21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>2</v>
+      </c>
+      <c r="B22">
+        <v>38</v>
+      </c>
+      <c r="C22">
+        <v>62</v>
+      </c>
+      <c r="D22">
+        <v>42</v>
+      </c>
+      <c r="E22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>6</v>
+      </c>
+      <c r="B23">
+        <v>66</v>
+      </c>
+      <c r="C23">
+        <v>85</v>
+      </c>
+      <c r="D23">
+        <v>75</v>
+      </c>
+      <c r="E23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>5</v>
+      </c>
+      <c r="B24">
+        <v>57</v>
+      </c>
+      <c r="C24">
+        <v>78</v>
+      </c>
+      <c r="D24">
+        <v>64</v>
+      </c>
+      <c r="E24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>7</v>
+      </c>
+      <c r="B25">
+        <v>70</v>
+      </c>
+      <c r="C25">
+        <v>90</v>
+      </c>
+      <c r="D25">
+        <v>82</v>
+      </c>
+      <c r="E25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>3</v>
+      </c>
+      <c r="B26">
+        <v>47</v>
+      </c>
+      <c r="C26">
+        <v>72</v>
+      </c>
+      <c r="D26">
+        <v>55</v>
+      </c>
+      <c r="E26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>4</v>
+      </c>
+      <c r="B27">
+        <v>53</v>
+      </c>
+      <c r="C27">
+        <v>76</v>
+      </c>
+      <c r="D27">
+        <v>58</v>
+      </c>
+      <c r="E27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>5</v>
+      </c>
+      <c r="B28">
+        <v>61</v>
+      </c>
+      <c r="C28">
+        <v>82</v>
+      </c>
+      <c r="D28">
+        <v>68</v>
+      </c>
+      <c r="E28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>7</v>
+      </c>
+      <c r="B29">
+        <v>70</v>
+      </c>
+      <c r="C29">
+        <v>90</v>
+      </c>
+      <c r="D29">
+        <v>82</v>
+      </c>
+      <c r="E29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>3</v>
+      </c>
+      <c r="B30">
+        <v>47</v>
+      </c>
+      <c r="C30">
+        <v>72</v>
+      </c>
+      <c r="D30">
+        <v>55</v>
+      </c>
+      <c r="E30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <v>4</v>
+      </c>
+      <c r="B31">
+        <v>53</v>
+      </c>
+      <c r="C31">
+        <v>76</v>
+      </c>
+      <c r="D31">
+        <v>58</v>
+      </c>
+      <c r="E31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>5</v>
+      </c>
+      <c r="B32">
+        <v>61</v>
+      </c>
+      <c r="C32">
+        <v>82</v>
+      </c>
+      <c r="D32">
+        <v>68</v>
+      </c>
+      <c r="E32">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <v>6</v>
+      </c>
+      <c r="B33">
+        <v>63</v>
+      </c>
+      <c r="C33">
+        <v>79</v>
+      </c>
+      <c r="D33">
+        <v>70</v>
+      </c>
+      <c r="E33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A34">
+        <v>2</v>
+      </c>
+      <c r="B34">
+        <v>36</v>
+      </c>
+      <c r="C34">
+        <v>58</v>
+      </c>
+      <c r="D34">
+        <v>40</v>
+      </c>
+      <c r="E34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A35">
+        <v>1</v>
+      </c>
+      <c r="B35">
+        <v>28</v>
+      </c>
+      <c r="C35">
+        <v>52</v>
+      </c>
+      <c r="D35">
+        <v>32</v>
+      </c>
+      <c r="E35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A36">
+        <v>8</v>
+      </c>
+      <c r="B36">
+        <v>82</v>
+      </c>
+      <c r="C36">
+        <v>91</v>
+      </c>
+      <c r="D36">
+        <v>85</v>
+      </c>
+      <c r="E36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A37">
+        <v>9</v>
+      </c>
+      <c r="B37">
+        <v>90</v>
+      </c>
+      <c r="C37">
+        <v>94</v>
+      </c>
+      <c r="D37">
+        <v>93</v>
+      </c>
+      <c r="E37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A38">
+        <v>7</v>
+      </c>
+      <c r="B38">
+        <v>69</v>
+      </c>
+      <c r="C38">
+        <v>88</v>
+      </c>
+      <c r="D38">
+        <v>79</v>
+      </c>
+      <c r="E38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A39">
+        <v>5</v>
+      </c>
+      <c r="B39">
+        <v>50</v>
+      </c>
+      <c r="C39">
+        <v>65</v>
+      </c>
+      <c r="D39">
+        <v>55</v>
+      </c>
+      <c r="E39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A40">
+        <v>4</v>
+      </c>
+      <c r="B40">
+        <v>60</v>
+      </c>
+      <c r="C40">
+        <v>68</v>
+      </c>
+      <c r="D40">
+        <v>62</v>
+      </c>
+      <c r="E40">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A41">
+        <v>3</v>
+      </c>
+      <c r="B41">
+        <v>44</v>
+      </c>
+      <c r="C41">
+        <v>70</v>
+      </c>
+      <c r="D41">
+        <v>52</v>
+      </c>
+      <c r="E41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A42">
+        <v>2</v>
+      </c>
+      <c r="B42">
+        <v>41</v>
+      </c>
+      <c r="C42">
+        <v>67</v>
+      </c>
+      <c r="D42">
+        <v>45</v>
+      </c>
+      <c r="E42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A43">
+        <v>6</v>
+      </c>
+      <c r="B43">
+        <v>71</v>
+      </c>
+      <c r="C43">
+        <v>83</v>
+      </c>
+      <c r="D43">
+        <v>77</v>
+      </c>
+      <c r="E43">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A44">
+        <v>7</v>
+      </c>
+      <c r="B44">
+        <v>74</v>
+      </c>
+      <c r="C44">
+        <v>86</v>
+      </c>
+      <c r="D44">
+        <v>81</v>
+      </c>
+      <c r="E44">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A45">
+        <v>8</v>
+      </c>
+      <c r="B45">
+        <v>79</v>
+      </c>
+      <c r="C45">
+        <v>89</v>
+      </c>
+      <c r="D45">
+        <v>84</v>
+      </c>
+      <c r="E45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A46">
+        <v>1</v>
+      </c>
+      <c r="B46">
+        <v>20</v>
+      </c>
+      <c r="C46">
+        <v>45</v>
+      </c>
+      <c r="D46">
+        <v>25</v>
+      </c>
+      <c r="E46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A47">
+        <v>2</v>
+      </c>
+      <c r="B47">
+        <v>32</v>
+      </c>
+      <c r="C47">
+        <v>55</v>
+      </c>
+      <c r="D47">
+        <v>35</v>
+      </c>
+      <c r="E47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A48">
+        <v>4</v>
+      </c>
+      <c r="B48">
+        <v>58</v>
+      </c>
+      <c r="C48">
+        <v>80</v>
+      </c>
+      <c r="D48">
+        <v>65</v>
+      </c>
+      <c r="E48">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A49">
+        <v>5</v>
+      </c>
+      <c r="B49">
+        <v>62</v>
+      </c>
+      <c r="C49">
+        <v>84</v>
+      </c>
+      <c r="D49">
+        <v>70</v>
+      </c>
+      <c r="E49">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A50">
+        <v>6</v>
+      </c>
+      <c r="B50">
+        <v>67</v>
+      </c>
+      <c r="C50">
+        <v>86</v>
+      </c>
+      <c r="D50">
+        <v>75</v>
+      </c>
+      <c r="E50">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A51">
+        <v>3</v>
+      </c>
+      <c r="B51">
+        <v>49</v>
+      </c>
+      <c r="C51">
+        <v>74</v>
+      </c>
+      <c r="D51">
+        <v>57</v>
+      </c>
+      <c r="E51">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A52">
+        <v>7</v>
+      </c>
+      <c r="B52">
+        <v>78</v>
+      </c>
+      <c r="C52">
+        <v>92</v>
+      </c>
+      <c r="D52">
+        <v>86</v>
+      </c>
+      <c r="E52">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A53">
+        <v>8</v>
+      </c>
+      <c r="B53">
+        <v>85</v>
+      </c>
+      <c r="C53">
+        <v>95</v>
+      </c>
+      <c r="D53">
+        <v>88</v>
+      </c>
+      <c r="E53">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A54">
+        <v>9</v>
+      </c>
+      <c r="B54">
+        <v>87</v>
+      </c>
+      <c r="C54">
+        <v>93</v>
+      </c>
+      <c r="D54">
+        <v>90</v>
+      </c>
+      <c r="E54">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A55">
+        <v>10</v>
+      </c>
+      <c r="B55">
+        <v>95</v>
+      </c>
+      <c r="C55">
+        <v>98</v>
+      </c>
+      <c r="D55">
+        <v>97</v>
+      </c>
+      <c r="E55">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>